<commit_message>
feat(config): 微信 AppID 落地 + 文档/设计稿口径升 v1.7 / v2.1
- broadband-miniapp/project.config.json：appid 由 touristappid 改为真实 wxcc344ad7f4f849d4
- backend application.yml：app.wechat.miniapp.appid 默认值回填该 AppID，Secret 仍走环境变量 WECHAT_SECRET
- docs/功能进度说明书.md（v1.7）：新增凭证与环境变量清单 5.1；修正师傅端 6 行过期接口口径（/api/admin/* → /api/worker/*，补数据隔离说明）；更新剩余缺口
- docs/项目进度与开发计划.xlsx（v1.7）：新增 AppID 落地行与「外部凭证」统计行；待办 #1 收敛为「注入 WECHAT_SECRET」，新增 #10 AppID 拆分确认；里程碑新增 M10b（Secret 接入）/ M10c（视觉验收）
- broadband-design/index.html（v2.1）：落地状态总览加「微信凭证 90%」行、新增凭证与环境变量表、师傅端页面清单对齐真实接口、后续计划刷新
- scripts/：归档 xlsx 与 md→docx 生成脚本，便于口径复现
</commit_message>
<xml_diff>
--- a/docs/项目进度与开发计划.xlsx
+++ b/docs/项目进度与开发计划.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -496,7 +496,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>生成日期 2026-09-14 ｜ 后端 4 模块+1公共层 / 56 接口 / 小程序 28 页 / PC后台 25 页 ｜ 口径版本 v1.6（M9 双端登录态收口 + M10 师傅端数据绑定与隔离 均已完成）</t>
+          <t>生成日期 2026-09-15 ｜ 后端 4 模块+1公共层 / 56 接口 / 小程序 28 页 / PC后台 25 页 ｜ 口径版本 v1.7（M9 双端登录态收口 + M10 师傅端数据绑定与隔离 已完成；微信 AppID 已就位，缺 AppSecret）</t>
         </is>
       </c>
     </row>
@@ -800,12 +800,12 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>后端 · C端鉴权收口（M9）</t>
+          <t>后端 · 微信 AppID 落地（M10）</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>protect-client-api=true，C 端接口强制校验 JWT</t>
+          <t>两端 project.config.json + 后端 application.yml 均写入真实 AppID</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -820,19 +820,19 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>JwtAuthFilter 新增 CUSTOMER 分支（CustomerPrincipal + ROLE_CUSTOMER）</t>
+          <t>AppID wxcc344ad7f4f849d4；AppSecret 仍由环境变量 WECHAT_SECRET 注入（未注入即走演示码回退）</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>后端 · 师傅端登录（M9新增）</t>
+          <t>后端 · C端鉴权收口（M9）</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>按 worker.phone 查表签发 WORKER 令牌</t>
+          <t>protect-client-api=true，C 端接口强制校验 JWT</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -847,19 +847,19 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>POST /api/auth/worker-login（permitAll）</t>
+          <t>JwtAuthFilter 新增 CUSTOMER 分支（CustomerPrincipal + ROLE_CUSTOMER）</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>后端 · WORKER 令牌鉴权（M9）</t>
+          <t>后端 · 师傅端登录（M9新增）</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>师傅令牌可访问工单/SLA 接口，与后台 RBAC 隔离</t>
+          <t>按 worker.phone 查表签发 WORKER 令牌</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -874,19 +874,19 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>WorkerPrincipal + ROLE_WORKER + workorder:view + sla:view</t>
+          <t>POST /api/auth/worker-login（permitAll）</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>后端 · 师傅端数据接口（M10新增）</t>
+          <t>后端 · WORKER 令牌鉴权（M9）</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>本人工单列表/详情 · 首页统计 · 容量看板 · 7天排班 · 完工提交</t>
+          <t>师傅令牌可访问工单/SLA 接口，与后台 RBAC 隔离</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -901,19 +901,19 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>WorkerController 6 接口 /api/worker/*；服务端按 token 隔离，忽略客户端 workerId 传参</t>
+          <t>WorkerPrincipal + ROLE_WORKER + workorder:view + sla:view</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>后端 · 数据库接入 MySQL</t>
+          <t>后端 · 师傅端数据接口（M10新增）</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>25表 · 种子数据 · 启动自动初始化 · 全部接口连库</t>
+          <t>本人工单列表/详情 · 首页统计 · 容量看板 · 7天排班 · 完工提交</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -928,19 +928,19 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>schema.sql + data.sql（幂等）；M9 增列 customer.openid / worker.phone</t>
+          <t>WorkerController 6 接口 /api/worker/*；服务端按 token 隔离，忽略客户端 workerId 传参</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>后端 · 统一请求/错误处理</t>
+          <t>后端 · 数据库接入 MySQL</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>非2xx一律reject（原静默吞错）；401 自动跳登录页</t>
+          <t>25表 · 种子数据 · 启动自动初始化 · 全部接口连库</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -955,19 +955,19 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>utils/api.js（客户端 + 师傅端）</t>
+          <t>schema.sql + data.sql（幂等）；M9 增列 customer.openid / worker.phone</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>客户端小程序 broadband-miniapp</t>
+          <t>后端 · 统一请求/错误处理</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>20页：首页/服务/套餐(详情,列表,升级)/小区查询/订单(地址,确认,列表,详情)/地址/流量/移机/自助/智慧家庭/评价/我的/设置/登录</t>
+          <t>非2xx一律reject（原静默吞错）；401 自动跳登录页</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -982,19 +982,19 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>蓝#2563eb；登录走真实 miniapp-login，401 门禁已接</t>
+          <t>utils/api.js（客户端 + 师傅端）</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>安装师傅端小程序 broadband-worker</t>
+          <t>客户端小程序 broadband-miniapp</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>8页：首页/工单/工单详情/完工确认/容量/排班/我的/登录</t>
+          <t>20页：首页/服务/套餐(详情,列表,升级)/小区查询/订单(地址,确认,列表,详情)/地址/流量/移机/自助/智慧家庭/评价/我的/设置/登录</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -1009,19 +1009,19 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>橙#ea580c；登录改调真实 worker-login（原 mock 已废）</t>
+          <t>蓝#2563eb；登录走真实 miniapp-login，401 门禁已接</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>PC后台 web-admin</t>
+          <t>安装师傅端小程序 broadband-worker</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>25页/22路由：仪表盘/套餐/小区/工单/派单/容量/SLA/流量/升级/RBAC/客户/评价/审计/监控</t>
+          <t>8页：首页/工单/工单详情/完工确认/容量/排班/我的/登录</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
@@ -1036,134 +1036,134 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Vue3+ElementPlus按需+Pinia；按钮级 v-perm；菜单由后端 /api/auth/me 动态渲染</t>
+          <t>橙#ea580c；登录改调真实 worker-login（原 mock 已废）</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
+          <t>PC后台 web-admin</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>25页/22路由：仪表盘/套餐/小区/工单/派单/容量/SLA/流量/升级/RBAC/客户/评价/审计/监控</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>✅ 已完成</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Vue3+ElementPlus按需+Pinia；按钮级 v-perm；菜单由后端 /api/auth/me 动态渲染</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>外部凭证与环境变量</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>AppID 已配置 / Secret 待注入；JWT 密钥、DB 凭据、C 端鉴权开关均已明确</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>🟡 90%</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>AppID wxcc344ad7f4f849d4（两端共用）；缺 WECHAT_SECRET 时自动回退演示码 1234</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
           <t>文档套件</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>5份说明书 v1.4 + 模块文档(README/SLA/PKG_TRAFFIC/RBAC) + 本进度计划表 v1.5</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>✅ 已完成</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>md + docx 已同步项目空间「文档」</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="7" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>5份说明书 + 模块文档 + 进度计划表 v1.7 + 设计稿 v2.1</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>✅ 已完成</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>md + docx + xlsx + html 已同步项目空间</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
         <is>
           <t>总体进度统计</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>维度</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>规划中</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr">
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>覆盖率</t>
         </is>
       </c>
-      <c r="E27" s="3" t="inlineStr">
+      <c r="E29" s="3" t="inlineStr">
         <is>
           <t>备注</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>后端业务模块</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>4 + 1公共层</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>community / install / product / system + common</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>后端 REST 接口</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>56（GET36 / POST15 / PUT5）</t>
-        </is>
-      </c>
-      <c r="C29" s="6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D29" s="6" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>M9 +worker-login（49→50）；M10 +6 个 /api/worker/*（50→56）</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>数据库表</t>
+          <t>后端业务模块</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>25 张 + 种子数据</t>
+          <t>4 + 1公共层</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -1178,19 +1178,19 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>M9 仅加列未加表</t>
+          <t>community / install / product / system + common</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>安全与鉴权</t>
+          <t>后端 REST 接口</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>5角色 / 26菜单 / 21权限码</t>
+          <t>56（GET36 / POST15 / PUT5）</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
@@ -1205,19 +1205,19 @@
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>M9 扩至 3 类令牌：SYS / CUSTOMER / WORKER</t>
+          <t>M9 +worker-login（49→50）；M10 +6 个 /api/worker/*（50→56）</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>客户端小程序页</t>
+          <t>数据库表</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>20（含登录页）</t>
+          <t>25 张 + 种子数据</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
@@ -1232,19 +1232,19 @@
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>设计稿 20 页全覆盖</t>
+          <t>M9 仅加列未加表</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>安装师傅端小程序页</t>
+          <t>安全与鉴权</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>8（含登录页）</t>
+          <t>5角色 / 26菜单 / 21权限码</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
@@ -1259,19 +1259,19 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>设计稿 8 页全覆盖</t>
+          <t>M9 扩至 3 类令牌：SYS / CUSTOMER / WORKER</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>PC 后台页面</t>
+          <t>客户端小程序页</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>25（22业务 + login + 403 + 404）</t>
+          <t>20（含登录页）</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
@@ -1286,34 +1286,88 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>设计稿 16 模块全覆盖</t>
+          <t>设计稿 20 页全覆盖</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
+          <t>安装师傅端小程序页</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>8（含登录页）</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>设计稿 8 页全覆盖</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>PC 后台页面</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>25（22业务 + login + 403 + 404）</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>设计稿 16 模块全覆盖</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
           <t>文档说明书</t>
         </is>
       </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>5 份 v1.4 + 进度计划表 v1.5</t>
-        </is>
-      </c>
-      <c r="C35" s="6" t="inlineStr">
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>说明书 v1.7（md/docx）+ 进度计划表 v1.7 + 设计稿 v2.1</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="D35" s="6" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="E35" s="4" t="inlineStr">
-        <is>
-          <t>md/docx/xlsx 三格式</t>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>md/docx/xlsx/html 四格式</t>
         </is>
       </c>
     </row>
@@ -1332,7 +1386,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1345,14 +1399,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>宽带业务管理系统 · 待开发功能清单（截至 2026-09-14，M9 收口后）</t>
+          <t>宽带业务管理系统 · 待开发功能清单（截至 2026-09-15，M10 收尾后）</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>说明：#1 已于 M9 完成并从待办移出；优先级为建议值，最终以负责人排期确认为准。</t>
+          <t>说明：原「微信真实凭证接入」已完成一半——AppID 已写入两端与后端配置，仅缺 AppSecret；优先级为建议值，最终以负责人排期确认为准。</t>
         </is>
       </c>
     </row>
@@ -1391,17 +1445,17 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>微信真实凭证接入（AppID/Secret）</t>
+          <t>微信 AppSecret 注入</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>双路径已就绪，当前走演示码 1234 回退</t>
+          <t>AppID 已配置（wxcc344ad7f4f849d4），登录仍走演示码 1234 回退</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>用户提供小程序 AppID + Secret 后，自动切换 code2Session 真实登录</t>
+          <t>提供 Secret 并导出环境变量 WECHAT_SECRET 后，自动切换 code2Session 真实登录，前端无需改动</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
@@ -1428,7 +1482,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>需微信开发者工具导入 broadband-worker 后截图验收（无浏览器环境）</t>
+          <t>需微信开发者工具导入 broadband-worker 后逐页截图验收（无浏览器环境）</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -1617,7 +1671,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>对齐设计稿 v1.9 剩余字段与图表</t>
+          <t>对齐设计稿 v2.1 剩余字段与图表</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
@@ -1634,20 +1688,47 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
+          <t>小程序 AppID 拆分（合规确认）</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>客户端与师傅端共用同一 AppID</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>提审前确认走「同主体多端」还是为师傅端单开 AppID</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
           <t>多端适配 / 国际化（可选）</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>未规划</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>视业务需要</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
@@ -1668,7 +1749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1689,7 +1770,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>M1–M9 为已完成里程碑；M10 起为建议排期（相对周次，需负责人确认后定稿）。</t>
+          <t>M1–M10 为已完成里程碑；M10b 起为建议排期（相对周次，需负责人确认后定稿）。代码已全量推送 GitHub（linxi072/broadband）。</t>
         </is>
       </c>
     </row>
@@ -2009,7 +2090,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>微信真实凭证待提供（当前演示码回退）</t>
+          <t>AppSecret 未注入，登录走演示码回退（AppID 已于 M10 补上）</t>
         </is>
       </c>
     </row>
@@ -2048,17 +2129,17 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>M10b 师傅端视觉验收</t>
+          <t>M10b 微信 AppSecret 接入</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>页面截图与交互验收</t>
+          <t>真实 code2Session 登录</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>微信开发者工具导入 broadband-worker 后逐页截图</t>
+          <t>导出 WECHAT_SECRET 环境变量，重启后端；验证 openid 落库与绑定客户</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -2068,29 +2149,29 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>建议 W1</t>
+          <t>随时（拿到 Secret 即刻）</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>无浏览器环境，需人工验收</t>
+          <t>Secret 属敏感项，不入库、不入文档</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>M11 业务闭环联调</t>
+          <t>M10c 师傅端视觉验收</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>下单→派单→装机→SLA→评价 端到端</t>
+          <t>页面截图与交互验收</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>订单状态机 · 派单回写 · SLA 赔付 · 评价落库</t>
+          <t>微信开发者工具导入 broadband-worker 后逐页截图</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -2100,29 +2181,29 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>建议 W2–W3</t>
+          <t>建议 W1</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>多状态一致性；支付可后置</t>
+          <t>无浏览器环境，需人工验收</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>M12 监控与配置治理</t>
+          <t>M11 业务闭环联调</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>可观测性 + 多环境配置</t>
+          <t>下单→派单→装机→SLA→评价 端到端</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>metrics/日志/告警 · 多环境 profile · 监控页接数</t>
+          <t>订单状态机 · 派单回写 · SLA 赔付 · 评价落库</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -2132,42 +2213,74 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>建议 W3–W4</t>
+          <t>建议 W2–W3</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>监控组件选型；不引入 Apollo 的边界</t>
+          <t>多状态一致性；支付可后置</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
+          <t>M12 监控与配置治理</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>可观测性 + 多环境配置</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>metrics/日志/告警 · 多环境 profile · 监控页接数</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>⬜ 规划中</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>建议 W3–W4</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>监控组件选型；不引入 Apollo 的边界</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
           <t>M13 CI/CD 与上线</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>自动化构建部署 + 文档收尾</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>CI 流水线 · 生产 Nginx 部署 · 文档终版 · 复盘</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>⬜ 规划中</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>建议 W4–W5</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>生产密钥管理（jwt.secret 走环境变量）；GitHub 推送待 SSH 恢复</t>
         </is>
@@ -2208,7 +2321,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>口径 v1.6（M9 + M10 后）：新增 POST /api/auth/worker-login 与 6 个 /api/worker/* 接口，全部接口连库可用。</t>
+          <t>口径 v1.7（M9 + M10 后）：新增 POST /api/auth/worker-login 与 6 个 /api/worker/* 接口；AppID wxcc344ad7f4f849d4 已回填，全部接口连库可用。</t>
         </is>
       </c>
     </row>

</xml_diff>